<commit_message>
Add Day 5 sorting algorithms implementation
</commit_message>
<xml_diff>
--- a/My personal Notes.xlsx
+++ b/My personal Notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GUVI HCL Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697CD713-6025-4382-B2B3-0A13B22789E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D883598-2D55-4B16-9740-F917E5809086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
+    <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="9960" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>Date</t>
   </si>
@@ -63,9 +63,6 @@
     <t>Day 1.docx</t>
   </si>
   <si>
-    <t>https://github.com/Suryaveera04/Guvi_Training_Day1.git</t>
-  </si>
-  <si>
     <t>Day 2</t>
   </si>
   <si>
@@ -85,6 +82,18 @@
   </si>
   <si>
     <t>Day 2.docx</t>
+  </si>
+  <si>
+    <t>https://github.com/Suryaveera04/GUVI_Training.git</t>
+  </si>
+  <si>
+    <t>Day 4</t>
+  </si>
+  <si>
+    <t>Day 4.docx</t>
+  </si>
+  <si>
+    <t>Two pointers, linear and binary search, Arrays, Strings</t>
   </si>
 </sst>
 </file>
@@ -461,12 +470,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47B9E310-7AC1-491F-A23C-6FB00D7310B7}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.21875" customWidth="1"/>
-    <col min="4" max="4" width="36.88671875" customWidth="1"/>
+    <col min="4" max="4" width="47.21875" customWidth="1"/>
     <col min="5" max="5" width="34.77734375" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="48.109375" customWidth="1"/>
@@ -509,7 +518,7 @@
         <v>8</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -517,15 +526,18 @@
         <v>46025</v>
       </c>
       <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
         <v>10</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>16</v>
       </c>
     </row>
@@ -534,13 +546,33 @@
         <v>46027</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>15</v>
+      <c r="G8" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B9" s="2">
+        <v>46028</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -552,8 +584,12 @@
     <hyperlink ref="E8" r:id="rId4" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQClqAX-T6dtSpRmdg1T-gDaAe34J8AqaeRn4jCj5s0N4No?e=wgkpZa" xr:uid="{909E0AED-7663-4D82-832E-10912654DC07}"/>
     <hyperlink ref="F8" r:id="rId5" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQAtbEYWy8nZQoQGlRnNfKI-AVECNx3-gk4ZlwRBghzy-lM?e=8Gmj47" xr:uid="{253ED195-8EBD-4ADC-9B2C-1A2A0119ECE9}"/>
     <hyperlink ref="F7" r:id="rId6" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQACI38hWtVSQIy0bmgAiEqsAYDazaHy7ZV1ehBlKeN4ZRs?e=7cdq83" xr:uid="{D78E377D-F5DA-47F9-B6D3-BBE541414887}"/>
+    <hyperlink ref="G7" r:id="rId7" xr:uid="{AA658E18-CD3E-4864-A5CD-B2DFC6189D59}"/>
+    <hyperlink ref="G8" r:id="rId8" xr:uid="{3F187B74-76CE-4E8F-9FB6-B02B8191734C}"/>
+    <hyperlink ref="F9" r:id="rId9" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQDHiH5GOAe_S7_7pIvaqYWsAetGbdz-d08pYJ4dmvBuMUw?e=K55StL" xr:uid="{0EF4F5F1-B0C2-4E65-B542-82D4201F11E0}"/>
+    <hyperlink ref="G9" r:id="rId10" xr:uid="{22678D11-0E42-483E-8B00-DFCA10BC6E88}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId7"/>
+  <pageSetup orientation="portrait" r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reorganize files and update training notes
</commit_message>
<xml_diff>
--- a/My personal Notes.xlsx
+++ b/My personal Notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GUVI HCL Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D883598-2D55-4B16-9740-F917E5809086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC26789-F80A-4A7B-A14D-448D743C6890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="9960" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Date</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t>Two pointers, linear and binary search, Arrays, Strings</t>
+  </si>
+  <si>
+    <t>Day 5</t>
+  </si>
+  <si>
+    <t>Oops Concepts, 54</t>
   </si>
 </sst>
 </file>
@@ -470,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47B9E310-7AC1-491F-A23C-6FB00D7310B7}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -548,6 +554,9 @@
       <c r="C8" t="s">
         <v>11</v>
       </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
       <c r="E8" s="3" t="s">
         <v>13</v>
       </c>
@@ -573,21 +582,29 @@
       </c>
       <c r="G9" s="3" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B10" s="2">
+        <v>46029</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="F6" r:id="rId1" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQB-bA3HXD49TaLw56hrq0czAY9dFEZRenF4QzCXFto557c?e=MtkT4H" xr:uid="{AEABD075-E105-4375-87B3-468F58B11AF9}"/>
-    <hyperlink ref="G6" r:id="rId2" xr:uid="{2B93A83E-F1D3-4B43-A1B2-35D276467E49}"/>
-    <hyperlink ref="E7" r:id="rId3" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQCDCvyev9_VRrUFU5em3_ZYAblpL9PFPsFmoNLJ8RayXqQ?e=yLOMLL" xr:uid="{3759B9C8-9425-4320-B501-9C000D77471E}"/>
-    <hyperlink ref="E8" r:id="rId4" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQClqAX-T6dtSpRmdg1T-gDaAe34J8AqaeRn4jCj5s0N4No?e=wgkpZa" xr:uid="{909E0AED-7663-4D82-832E-10912654DC07}"/>
-    <hyperlink ref="F8" r:id="rId5" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQAtbEYWy8nZQoQGlRnNfKI-AVECNx3-gk4ZlwRBghzy-lM?e=8Gmj47" xr:uid="{253ED195-8EBD-4ADC-9B2C-1A2A0119ECE9}"/>
-    <hyperlink ref="F7" r:id="rId6" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQACI38hWtVSQIy0bmgAiEqsAYDazaHy7ZV1ehBlKeN4ZRs?e=7cdq83" xr:uid="{D78E377D-F5DA-47F9-B6D3-BBE541414887}"/>
-    <hyperlink ref="G7" r:id="rId7" xr:uid="{AA658E18-CD3E-4864-A5CD-B2DFC6189D59}"/>
-    <hyperlink ref="G8" r:id="rId8" xr:uid="{3F187B74-76CE-4E8F-9FB6-B02B8191734C}"/>
-    <hyperlink ref="F9" r:id="rId9" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQDHiH5GOAe_S7_7pIvaqYWsAetGbdz-d08pYJ4dmvBuMUw?e=K55StL" xr:uid="{0EF4F5F1-B0C2-4E65-B542-82D4201F11E0}"/>
-    <hyperlink ref="G9" r:id="rId10" xr:uid="{22678D11-0E42-483E-8B00-DFCA10BC6E88}"/>
+    <hyperlink ref="E7" r:id="rId2" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQCDCvyev9_VRrUFU5em3_ZYAblpL9PFPsFmoNLJ8RayXqQ?e=yLOMLL" xr:uid="{3759B9C8-9425-4320-B501-9C000D77471E}"/>
+    <hyperlink ref="E8" r:id="rId3" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQClqAX-T6dtSpRmdg1T-gDaAe34J8AqaeRn4jCj5s0N4No?e=wgkpZa" xr:uid="{909E0AED-7663-4D82-832E-10912654DC07}"/>
+    <hyperlink ref="F8" r:id="rId4" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQAtbEYWy8nZQoQGlRnNfKI-AVECNx3-gk4ZlwRBghzy-lM?e=8Gmj47" xr:uid="{253ED195-8EBD-4ADC-9B2C-1A2A0119ECE9}"/>
+    <hyperlink ref="F7" r:id="rId5" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQACI38hWtVSQIy0bmgAiEqsAYDazaHy7ZV1ehBlKeN4ZRs?e=7cdq83" xr:uid="{D78E377D-F5DA-47F9-B6D3-BBE541414887}"/>
+    <hyperlink ref="G7" r:id="rId6" xr:uid="{AA658E18-CD3E-4864-A5CD-B2DFC6189D59}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{3F187B74-76CE-4E8F-9FB6-B02B8191734C}"/>
+    <hyperlink ref="F9" r:id="rId8" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQDHiH5GOAe_S7_7pIvaqYWsAetGbdz-d08pYJ4dmvBuMUw?e=K55StL" xr:uid="{0EF4F5F1-B0C2-4E65-B542-82D4201F11E0}"/>
+    <hyperlink ref="G9" r:id="rId9" xr:uid="{22678D11-0E42-483E-8B00-DFCA10BC6E88}"/>
+    <hyperlink ref="G6" r:id="rId10" xr:uid="{2B93A83E-F1D3-4B43-A1B2-35D276467E49}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId11"/>

</xml_diff>

<commit_message>
Update training notes with latest progress
</commit_message>
<xml_diff>
--- a/My personal Notes.xlsx
+++ b/My personal Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GUVI HCL Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC26789-F80A-4A7B-A14D-448D743C6890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF225BCB-55A2-42D5-BEB7-68DE0AEFEB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -100,6 +100,15 @@
   </si>
   <si>
     <t>Oops Concepts, 54</t>
+  </si>
+  <si>
+    <t>Ternary Search, Bubble sort, Insertion Sort, Selection sort</t>
+  </si>
+  <si>
+    <t>Day 6</t>
+  </si>
+  <si>
+    <t>Quick Sort, Merge sort, Bucket sort</t>
   </si>
 </sst>
 </file>
@@ -476,12 +485,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47B9E310-7AC1-491F-A23C-6FB00D7310B7}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.21875" customWidth="1"/>
-    <col min="4" max="4" width="47.21875" customWidth="1"/>
+    <col min="4" max="4" width="50.44140625" customWidth="1"/>
     <col min="5" max="5" width="34.77734375" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="48.109375" customWidth="1"/>
@@ -590,6 +599,26 @@
       </c>
       <c r="C10" t="s">
         <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B11" s="2">
+        <v>46030</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -605,8 +634,10 @@
     <hyperlink ref="F9" r:id="rId8" display="https://1drv.ms/w/c/9b312b9e72a46ecf/IQDHiH5GOAe_S7_7pIvaqYWsAetGbdz-d08pYJ4dmvBuMUw?e=K55StL" xr:uid="{0EF4F5F1-B0C2-4E65-B542-82D4201F11E0}"/>
     <hyperlink ref="G9" r:id="rId9" xr:uid="{22678D11-0E42-483E-8B00-DFCA10BC6E88}"/>
     <hyperlink ref="G6" r:id="rId10" xr:uid="{2B93A83E-F1D3-4B43-A1B2-35D276467E49}"/>
+    <hyperlink ref="G10" r:id="rId11" xr:uid="{339A4775-B4E9-4438-A7D1-7213384182A6}"/>
+    <hyperlink ref="G11" r:id="rId12" xr:uid="{A8A78672-A2FC-403D-A24B-6F059CBECA52}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId11"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix binary search logic in situation3.java and sliding window in subarray.java
</commit_message>
<xml_diff>
--- a/My personal Notes.xlsx
+++ b/My personal Notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GUVI HCL Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF225BCB-55A2-42D5-BEB7-68DE0AEFEB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EE9955-530E-469F-B344-F9BF341A5FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
+    <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="9960" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -96,9 +96,6 @@
     <t>Two pointers, linear and binary search, Arrays, Strings</t>
   </si>
   <si>
-    <t>Day 5</t>
-  </si>
-  <si>
     <t>Oops Concepts, 54</t>
   </si>
   <si>
@@ -109,6 +106,21 @@
   </si>
   <si>
     <t>Quick Sort, Merge sort, Bucket sort</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Radix sort, Time complexity</t>
+  </si>
+  <si>
+    <t>Day 5-2</t>
+  </si>
+  <si>
+    <t>Day 5-1</t>
+  </si>
+  <si>
+    <t>Day 8</t>
+  </si>
+  <si>
+    <t>Binary Search(leetcode Problems) twopointer sum(subarray, subset)</t>
   </si>
 </sst>
 </file>
@@ -485,12 +497,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47B9E310-7AC1-491F-A23C-6FB00D7310B7}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.21875" customWidth="1"/>
-    <col min="4" max="4" width="50.44140625" customWidth="1"/>
+    <col min="4" max="4" width="57.6640625" customWidth="1"/>
     <col min="5" max="5" width="34.77734375" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="48.109375" customWidth="1"/>
@@ -564,7 +576,7 @@
         <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>13</v>
@@ -598,10 +610,10 @@
         <v>46029</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>16</v>
@@ -612,13 +624,35 @@
         <v>46030</v>
       </c>
       <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s">
         <v>23</v>
-      </c>
-      <c r="D11" t="s">
-        <v>24</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" s="2">
+        <v>46031</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B13" s="2">
+        <v>46041</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Day 7 content and clean up Day 8 files
</commit_message>
<xml_diff>
--- a/My personal Notes.xlsx
+++ b/My personal Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GUVI HCL Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EE9955-530E-469F-B344-F9BF341A5FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C55473-B848-46EC-90DB-7C4CA926E2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="9960" xr2:uid="{9F942106-FAFB-473F-BB20-53478CADE758}"/>
   </bookViews>
@@ -117,10 +117,10 @@
     <t>Day 5-1</t>
   </si>
   <si>
-    <t>Day 8</t>
-  </si>
-  <si>
     <t>Binary Search(leetcode Problems) twopointer sum(subarray, subset)</t>
+  </si>
+  <si>
+    <t>Day 7</t>
   </si>
 </sst>
 </file>
@@ -649,10 +649,10 @@
         <v>46041</v>
       </c>
       <c r="C13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" t="s">
         <v>27</v>
-      </c>
-      <c r="D13" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>